<commit_message>
mostly State of Health Report work
</commit_message>
<xml_diff>
--- a/myAnalyses/0.StateOfHealth/Age Adjustment Explore.xlsx
+++ b/myAnalyses/0.StateOfHealth/Age Adjustment Explore.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\0.CBD\myAnalyses\0.StateOfHealth\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="120" yWindow="150" windowWidth="7635" windowHeight="9540"/>
+    <workbookView xWindow="120" yWindow="150" windowWidth="7635" windowHeight="9540" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="raceAgetemp" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="30">
   <si>
     <t>sex</t>
   </si>
@@ -86,18 +92,37 @@
   </si>
   <si>
     <t>ADJUSTED</t>
+  </si>
+  <si>
+    <t>Age Group</t>
+  </si>
+  <si>
+    <t>Total:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Crude</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Age-Adjusted</t>
+  </si>
+  <si>
+    <t>Black and White All-Cause Age-Specific Death Rates, and Rate Ratios</t>
+  </si>
+  <si>
+    <t>California 2016-2018</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0.0_);_(* \(#,##0.0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,6 +258,28 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="33">
     <fill>
@@ -415,7 +462,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -530,6 +577,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -576,7 +660,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -584,6 +668,35 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="18" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -638,6 +751,9 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
@@ -685,7 +801,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -720,7 +836,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1002,11 +1118,11 @@
         <v>2077497.528803</v>
       </c>
       <c r="K2" s="3">
-        <f>D2*100000/G2</f>
+        <f t="shared" ref="K2:K11" si="0">D2*100000/G2</f>
         <v>190.8713914504188</v>
       </c>
       <c r="L2" s="3">
-        <f>E2*100000/H2</f>
+        <f t="shared" ref="L2:L11" si="1">E2*100000/H2</f>
         <v>73.694431823566234</v>
       </c>
       <c r="N2" s="1">
@@ -1017,7 +1133,7 @@
         <v>18987</v>
       </c>
       <c r="Q2" s="5">
-        <f>P2*(D2/G2)</f>
+        <f t="shared" ref="Q2:Q11" si="2">P2*(D2/G2)</f>
         <v>36.240751094691014</v>
       </c>
     </row>
@@ -1041,11 +1157,11 @@
         <v>4031885.841428</v>
       </c>
       <c r="K3" s="3">
-        <f>D3*100000/G3</f>
+        <f t="shared" si="0"/>
         <v>18.018884048200437</v>
       </c>
       <c r="L3" s="3">
-        <f>E3*100000/H3</f>
+        <f t="shared" si="1"/>
         <v>9.2016494164576947</v>
       </c>
       <c r="N3" s="1">
@@ -1056,7 +1172,7 @@
         <v>39977</v>
       </c>
       <c r="Q3" s="5">
-        <f>P3*(D3/G3)</f>
+        <f t="shared" si="2"/>
         <v>7.2034092759490891</v>
       </c>
     </row>
@@ -1080,22 +1196,22 @@
         <v>4729163.6051829997</v>
       </c>
       <c r="K4" s="3">
-        <f>D4*100000/G4</f>
+        <f t="shared" si="0"/>
         <v>100.19040161123772</v>
       </c>
       <c r="L4" s="3">
-        <f>E4*100000/H4</f>
+        <f t="shared" si="1"/>
         <v>52.863470345159691</v>
       </c>
       <c r="N4" s="1">
-        <f t="shared" ref="N4:N15" si="0">K4/L4</f>
+        <f t="shared" ref="N4:N15" si="3">K4/L4</f>
         <v>1.8952672035541345</v>
       </c>
       <c r="P4">
         <v>38077</v>
       </c>
       <c r="Q4" s="5">
-        <f>P4*(D4/G4)</f>
+        <f t="shared" si="2"/>
         <v>38.149499221510986</v>
       </c>
     </row>
@@ -1119,22 +1235,22 @@
         <v>5496506.0594119998</v>
       </c>
       <c r="K5" s="3">
-        <f>D5*100000/G5</f>
+        <f t="shared" si="0"/>
         <v>167.17115326818109</v>
       </c>
       <c r="L5" s="3">
-        <f>E5*100000/H5</f>
+        <f t="shared" si="1"/>
         <v>102.48328554744833</v>
       </c>
       <c r="N5" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1.6312040775740271</v>
       </c>
       <c r="P5">
         <v>37233</v>
       </c>
       <c r="Q5" s="5">
-        <f>P5*(D5/G5)</f>
+        <f t="shared" si="2"/>
         <v>62.242835496341868</v>
       </c>
     </row>
@@ -1158,22 +1274,22 @@
         <v>5356504.9367119996</v>
       </c>
       <c r="K6" s="3">
-        <f>D6*100000/G6</f>
+        <f t="shared" si="0"/>
         <v>275.67166901520471</v>
       </c>
       <c r="L6" s="3">
-        <f>E6*100000/H6</f>
+        <f t="shared" si="1"/>
         <v>148.39900446128144</v>
       </c>
       <c r="N6" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1.857638263921978</v>
       </c>
       <c r="P6">
         <v>44659</v>
       </c>
       <c r="Q6" s="5">
-        <f>P6*(D6/G6)</f>
+        <f t="shared" si="2"/>
         <v>123.11221066550026</v>
       </c>
     </row>
@@ -1197,22 +1313,22 @@
         <v>6232040.5819429997</v>
       </c>
       <c r="K7" s="3">
-        <f>D7*100000/G7</f>
+        <f t="shared" si="0"/>
         <v>564.05496424190176</v>
       </c>
       <c r="L7" s="3">
-        <f>E7*100000/H7</f>
+        <f t="shared" si="1"/>
         <v>341.99071266886909</v>
       </c>
       <c r="N7" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1.6493283102341008</v>
       </c>
       <c r="P7">
         <v>37030</v>
       </c>
       <c r="Q7" s="5">
-        <f>P7*(D7/G7)</f>
+        <f t="shared" si="2"/>
         <v>208.86955325877625</v>
       </c>
     </row>
@@ -1236,22 +1352,22 @@
         <v>7277768.1993800001</v>
       </c>
       <c r="K8" s="3">
-        <f>D8*100000/G8</f>
+        <f t="shared" si="0"/>
         <v>1277.670228735765</v>
       </c>
       <c r="L8" s="3">
-        <f>E8*100000/H8</f>
+        <f t="shared" si="1"/>
         <v>750.93075930414727</v>
       </c>
       <c r="N8" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1.7014487859303071</v>
       </c>
       <c r="P8">
         <v>23961</v>
       </c>
       <c r="Q8" s="5">
-        <f>P8*(D8/G8)</f>
+        <f t="shared" si="2"/>
         <v>306.14256350737662</v>
       </c>
     </row>
@@ -1275,22 +1391,22 @@
         <v>5587305.9536739998</v>
       </c>
       <c r="K9" s="3">
-        <f>D9*100000/G9</f>
+        <f t="shared" si="0"/>
         <v>2450.0995503452637</v>
       </c>
       <c r="L9" s="3">
-        <f>E9*100000/H9</f>
+        <f t="shared" si="1"/>
         <v>1543.2840212249296</v>
       </c>
       <c r="N9" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1.5875882317504848</v>
       </c>
       <c r="P9">
         <v>18136</v>
       </c>
       <c r="Q9" s="5">
-        <f>P9*(D9/G9)</f>
+        <f t="shared" si="2"/>
         <v>444.35005445061705</v>
       </c>
     </row>
@@ -1314,22 +1430,22 @@
         <v>2778066.3869039998</v>
       </c>
       <c r="K10" s="3">
-        <f>D10*100000/G10</f>
+        <f t="shared" si="0"/>
         <v>5000.9672281315952</v>
       </c>
       <c r="L10" s="3">
-        <f>E10*100000/H10</f>
+        <f t="shared" si="1"/>
         <v>4122.0757192782376</v>
       </c>
       <c r="N10" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1.2132157603857041</v>
       </c>
       <c r="P10">
         <v>12315</v>
       </c>
       <c r="Q10" s="5">
-        <f>P10*(D10/G10)</f>
+        <f t="shared" si="2"/>
         <v>615.86911414440601</v>
       </c>
     </row>
@@ -1353,22 +1469,22 @@
         <v>1359183.2075157301</v>
       </c>
       <c r="K11" s="3">
-        <f>D11*100000/G11</f>
+        <f t="shared" si="0"/>
         <v>11412.716607288887</v>
       </c>
       <c r="L11" s="3">
-        <f>E11*100000/H11</f>
+        <f t="shared" si="1"/>
         <v>13776.141359356296</v>
       </c>
       <c r="N11" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.82844073021490527</v>
       </c>
       <c r="P11">
         <v>4259</v>
       </c>
       <c r="Q11" s="5">
-        <f>P11*(D11/G11)</f>
+        <f t="shared" si="2"/>
         <v>486.06760030443365</v>
       </c>
     </row>
@@ -1416,7 +1532,7 @@
         <v>1072.7281162344848</v>
       </c>
       <c r="N13" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.82479579443337903</v>
       </c>
       <c r="P13">
@@ -1445,7 +1561,7 @@
         <v>663.8</v>
       </c>
       <c r="N15" s="1">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>1.2771919252786985</v>
       </c>
       <c r="Q15" s="5">
@@ -1543,4 +1659,836 @@
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:V18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" customWidth="1"/>
+    <col min="3" max="3" width="1.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17.7109375" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5703125" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="5.28515625" customWidth="1"/>
+    <col min="7" max="8" width="20.7109375" customWidth="1"/>
+    <col min="9" max="10" width="18.5703125" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="2.7109375" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5703125" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="14.42578125" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="1.7109375" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" hidden="1" customWidth="1"/>
+    <col min="16" max="17" width="0" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="2.85546875" customWidth="1"/>
+    <col min="19" max="19" width="13.85546875" style="1" customWidth="1"/>
+    <col min="21" max="21" width="13.28515625" hidden="1" customWidth="1"/>
+    <col min="22" max="22" width="14.28515625" hidden="1" customWidth="1"/>
+    <col min="23" max="23" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="S1"/>
+    </row>
+    <row r="2" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="A2" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="S2"/>
+    </row>
+    <row r="4" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B4" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="8"/>
+      <c r="G4" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
+      <c r="L4" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="M4" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="N4" s="13"/>
+      <c r="O4" s="13"/>
+      <c r="P4" s="13"/>
+      <c r="Q4" s="13"/>
+      <c r="R4" s="13"/>
+      <c r="S4" s="29" t="s">
+        <v>19</v>
+      </c>
+      <c r="U4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B5" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="8"/>
+      <c r="D5" s="9">
+        <v>726</v>
+      </c>
+      <c r="E5" s="9">
+        <v>1531</v>
+      </c>
+      <c r="F5" s="9"/>
+      <c r="G5" s="15">
+        <f t="shared" ref="G5:G14" si="0">D5*100000/L5</f>
+        <v>190.8713914504188</v>
+      </c>
+      <c r="H5" s="15">
+        <f t="shared" ref="H5:H14" si="1">E5*100000/M5</f>
+        <v>73.694431823566234</v>
+      </c>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="11">
+        <v>380360.82541400002</v>
+      </c>
+      <c r="M5" s="11">
+        <v>2077497.528803</v>
+      </c>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+      <c r="R5" s="8"/>
+      <c r="S5" s="18">
+        <f t="shared" ref="S5:S14" si="2">G5/H5</f>
+        <v>2.5900381715051277</v>
+      </c>
+      <c r="U5">
+        <v>18987</v>
+      </c>
+      <c r="V5" s="5">
+        <f t="shared" ref="V5:V14" si="3">U5*(D5/L5)</f>
+        <v>36.240751094691014</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B6" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="8"/>
+      <c r="D6" s="9">
+        <v>143</v>
+      </c>
+      <c r="E6" s="9">
+        <v>371</v>
+      </c>
+      <c r="F6" s="9"/>
+      <c r="G6" s="16">
+        <f t="shared" si="0"/>
+        <v>18.018884048200437</v>
+      </c>
+      <c r="H6" s="16">
+        <f t="shared" si="1"/>
+        <v>9.2016494164576947</v>
+      </c>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="11">
+        <v>793611.85530399997</v>
+      </c>
+      <c r="M6" s="11">
+        <v>4031885.841428</v>
+      </c>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
+      <c r="R6" s="8"/>
+      <c r="S6" s="19">
+        <f t="shared" si="2"/>
+        <v>1.9582232741852343</v>
+      </c>
+      <c r="U6">
+        <v>39977</v>
+      </c>
+      <c r="V6" s="5">
+        <f t="shared" si="3"/>
+        <v>7.2034092759490891</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="8"/>
+      <c r="D7" s="9">
+        <v>980</v>
+      </c>
+      <c r="E7" s="9">
+        <v>2500</v>
+      </c>
+      <c r="F7" s="9"/>
+      <c r="G7" s="16">
+        <f t="shared" si="0"/>
+        <v>100.19040161123772</v>
+      </c>
+      <c r="H7" s="16">
+        <f t="shared" si="1"/>
+        <v>52.863470345159691</v>
+      </c>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="11">
+        <v>978137.61022999999</v>
+      </c>
+      <c r="M7" s="11">
+        <v>4729163.6051829997</v>
+      </c>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="19">
+        <f t="shared" si="2"/>
+        <v>1.8952672035541345</v>
+      </c>
+      <c r="U7">
+        <v>38077</v>
+      </c>
+      <c r="V7" s="5">
+        <f t="shared" si="3"/>
+        <v>38.149499221510986</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B8" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="8"/>
+      <c r="D8" s="9">
+        <v>1723</v>
+      </c>
+      <c r="E8" s="9">
+        <v>5633</v>
+      </c>
+      <c r="F8" s="9"/>
+      <c r="G8" s="16">
+        <f t="shared" si="0"/>
+        <v>167.17115326818109</v>
+      </c>
+      <c r="H8" s="16">
+        <f t="shared" si="1"/>
+        <v>102.48328554744833</v>
+      </c>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="11">
+        <v>1030680.2138499999</v>
+      </c>
+      <c r="M8" s="11">
+        <v>5496506.0594119998</v>
+      </c>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+      <c r="R8" s="8"/>
+      <c r="S8" s="19">
+        <f t="shared" si="2"/>
+        <v>1.6312040775740271</v>
+      </c>
+      <c r="U8">
+        <v>37233</v>
+      </c>
+      <c r="V8" s="5">
+        <f t="shared" si="3"/>
+        <v>62.242835496341868</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="8"/>
+      <c r="D9" s="9">
+        <v>2373</v>
+      </c>
+      <c r="E9" s="9">
+        <v>7949</v>
+      </c>
+      <c r="F9" s="9"/>
+      <c r="G9" s="16">
+        <f t="shared" si="0"/>
+        <v>275.67166901520471</v>
+      </c>
+      <c r="H9" s="16">
+        <f t="shared" si="1"/>
+        <v>148.39900446128144</v>
+      </c>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="11">
+        <v>860806.62858000002</v>
+      </c>
+      <c r="M9" s="11">
+        <v>5356504.9367119996</v>
+      </c>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
+      <c r="R9" s="8"/>
+      <c r="S9" s="19">
+        <f t="shared" si="2"/>
+        <v>1.857638263921978</v>
+      </c>
+      <c r="U9">
+        <v>44659</v>
+      </c>
+      <c r="V9" s="5">
+        <f t="shared" si="3"/>
+        <v>123.11221066550026</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B10" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="8"/>
+      <c r="D10" s="9">
+        <v>5341</v>
+      </c>
+      <c r="E10" s="9">
+        <v>21313</v>
+      </c>
+      <c r="F10" s="9"/>
+      <c r="G10" s="16">
+        <f t="shared" si="0"/>
+        <v>564.05496424190176</v>
+      </c>
+      <c r="H10" s="16">
+        <f t="shared" si="1"/>
+        <v>341.99071266886909</v>
+      </c>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="11">
+        <v>946893.53672800004</v>
+      </c>
+      <c r="M10" s="11">
+        <v>6232040.5819429997</v>
+      </c>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
+      <c r="R10" s="8"/>
+      <c r="S10" s="19">
+        <f t="shared" si="2"/>
+        <v>1.6493283102341008</v>
+      </c>
+      <c r="U10">
+        <v>37030</v>
+      </c>
+      <c r="V10" s="5">
+        <f t="shared" si="3"/>
+        <v>208.86955325877625</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B11" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="8"/>
+      <c r="D11" s="9">
+        <v>11576</v>
+      </c>
+      <c r="E11" s="9">
+        <v>54651</v>
+      </c>
+      <c r="F11" s="9"/>
+      <c r="G11" s="16">
+        <f t="shared" si="0"/>
+        <v>1277.670228735765</v>
+      </c>
+      <c r="H11" s="16">
+        <f t="shared" si="1"/>
+        <v>750.93075930414727</v>
+      </c>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="11">
+        <v>906024.08506099996</v>
+      </c>
+      <c r="M11" s="11">
+        <v>7277768.1993800001</v>
+      </c>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="19">
+        <f t="shared" si="2"/>
+        <v>1.7014487859303071</v>
+      </c>
+      <c r="U11">
+        <v>23961</v>
+      </c>
+      <c r="V11" s="5">
+        <f t="shared" si="3"/>
+        <v>306.14256350737662</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B12" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="8"/>
+      <c r="D12" s="9">
+        <v>12895</v>
+      </c>
+      <c r="E12" s="9">
+        <v>86228</v>
+      </c>
+      <c r="F12" s="9"/>
+      <c r="G12" s="16">
+        <f t="shared" si="0"/>
+        <v>2450.0995503452637</v>
+      </c>
+      <c r="H12" s="16">
+        <f t="shared" si="1"/>
+        <v>1543.2840212249296</v>
+      </c>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="11">
+        <v>526305.14536369999</v>
+      </c>
+      <c r="M12" s="11">
+        <v>5587305.9536739998</v>
+      </c>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8"/>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="19">
+        <f t="shared" si="2"/>
+        <v>1.5875882317504848</v>
+      </c>
+      <c r="U12">
+        <v>18136</v>
+      </c>
+      <c r="V12" s="5">
+        <f t="shared" si="3"/>
+        <v>444.35005445061705</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B13" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="8"/>
+      <c r="D13" s="9">
+        <v>12522</v>
+      </c>
+      <c r="E13" s="9">
+        <v>114514</v>
+      </c>
+      <c r="F13" s="9"/>
+      <c r="G13" s="16">
+        <f t="shared" si="0"/>
+        <v>5000.9672281315952</v>
+      </c>
+      <c r="H13" s="16">
+        <f t="shared" si="1"/>
+        <v>4122.0757192782376</v>
+      </c>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="11">
+        <v>250391.5628473</v>
+      </c>
+      <c r="M13" s="11">
+        <v>2778066.3869039998</v>
+      </c>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="19">
+        <f t="shared" si="2"/>
+        <v>1.2132157603857041</v>
+      </c>
+      <c r="U13">
+        <v>12315</v>
+      </c>
+      <c r="V13" s="5">
+        <f t="shared" si="3"/>
+        <v>615.86911414440601</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B14" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="8"/>
+      <c r="D14" s="9">
+        <v>11669</v>
+      </c>
+      <c r="E14" s="9">
+        <v>187243</v>
+      </c>
+      <c r="F14" s="9"/>
+      <c r="G14" s="17">
+        <f t="shared" si="0"/>
+        <v>11412.716607288887</v>
+      </c>
+      <c r="H14" s="17">
+        <f t="shared" si="1"/>
+        <v>13776.141359356296</v>
+      </c>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="11">
+        <v>102245.59499311</v>
+      </c>
+      <c r="M14" s="11">
+        <v>1359183.2075157301</v>
+      </c>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="20">
+        <f t="shared" si="2"/>
+        <v>0.82844073021490527</v>
+      </c>
+      <c r="U14">
+        <v>4259</v>
+      </c>
+      <c r="V14" s="5">
+        <f t="shared" si="3"/>
+        <v>486.06760030443365</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" ht="6" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="8"/>
+      <c r="S15" s="28"/>
+      <c r="V15" s="5"/>
+    </row>
+    <row r="16" spans="1:22" ht="21" x14ac:dyDescent="0.35">
+      <c r="B16" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="8"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="11"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="8"/>
+      <c r="R16" s="8"/>
+      <c r="S16" s="12"/>
+      <c r="V16" s="5"/>
+    </row>
+    <row r="17" spans="2:22" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B17" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="21"/>
+      <c r="D17" s="22">
+        <f>SUM(D5:D14)</f>
+        <v>59948</v>
+      </c>
+      <c r="E17" s="22">
+        <f>SUM(E5:E14)</f>
+        <v>481933</v>
+      </c>
+      <c r="F17" s="22"/>
+      <c r="G17" s="23">
+        <f>D17*100000/L17</f>
+        <v>884.78163884064406</v>
+      </c>
+      <c r="H17" s="23">
+        <f>E17*100000/M17</f>
+        <v>1072.7281162344848</v>
+      </c>
+      <c r="I17" s="22"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="L17" s="24">
+        <f>SUM(L5:L14)</f>
+        <v>6775457.0583711099</v>
+      </c>
+      <c r="M17" s="24">
+        <f>SUM(M5:M14)</f>
+        <v>44925922.300954729</v>
+      </c>
+      <c r="N17" s="21" t="s">
+        <v>17</v>
+      </c>
+      <c r="O17" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="P17" s="21"/>
+      <c r="Q17" s="21"/>
+      <c r="R17" s="21"/>
+      <c r="S17" s="26">
+        <f>G17/H17</f>
+        <v>0.82479579443337903</v>
+      </c>
+      <c r="U17">
+        <f>SUM(U5:U14)</f>
+        <v>274634</v>
+      </c>
+      <c r="V17" s="5">
+        <f>SUM(V5:V14)</f>
+        <v>2328.2475914196029</v>
+      </c>
+    </row>
+    <row r="18" spans="2:22" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B18" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="26">
+        <v>847.8</v>
+      </c>
+      <c r="H18" s="26">
+        <v>663.8</v>
+      </c>
+      <c r="I18" s="21"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="21"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="21"/>
+      <c r="N18" s="21"/>
+      <c r="O18" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="P18" s="21"/>
+      <c r="Q18" s="21"/>
+      <c r="R18" s="21"/>
+      <c r="S18" s="26">
+        <f>G18/H18</f>
+        <v>1.2771919252786985</v>
+      </c>
+      <c r="V18" s="5">
+        <f>V17*100000/U17</f>
+        <v>847.76378431643673</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="G5:H15">
+    <cfRule type="dataBar" priority="2">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{67FB8FF8-8789-4EEC-B0F0-88BBD4DF3C71}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S5:S15">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{9D913DAB-28C7-45AC-BE37-39A5A4B4FF0D}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U5:U16">
+    <cfRule type="dataBar" priority="7">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{A1562ED0-F0D1-4FBB-9F4B-58F2CBAD24D3}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L5:L16">
+    <cfRule type="dataBar" priority="9">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{F4C9CB50-678D-4202-95F2-4CA6F03289CD}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M5:M16">
+    <cfRule type="dataBar" priority="11">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF008AEF"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{BBF32305-7CDF-4443-83C4-B4012FBB0E2B}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{67FB8FF8-8789-4EEC-B0F0-88BBD4DF3C71}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF63C384"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>G5:H15</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{9D913DAB-28C7-45AC-BE37-39A5A4B4FF0D}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF008AEF"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>S5:S15</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{A1562ED0-F0D1-4FBB-9F4B-58F2CBAD24D3}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF008AEF"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>U5:U16</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{F4C9CB50-678D-4202-95F2-4CA6F03289CD}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF008AEF"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>L5:L16</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{BBF32305-7CDF-4443-83C4-B4012FBB0E2B}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FF008AEF"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>M5:M16</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>